<commit_message>
fix: reset all initial transactions to 0 and persist empty state until receipt is scanned
</commit_message>
<xml_diff>
--- a/ABA_Transactions_Latest.xlsx
+++ b/ABA_Transactions_Latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,94 +477,6 @@
           <t>Balance</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>09-Sep-2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>57550</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>JV00596</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>ខួបកំណើតនិងនំខេក បងវុធ</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>240000</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>57551</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>JV00597</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>ម៉ាយ ណាយ (Khmer Express)</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>ថ្លៃសេវាកម្មទូទៅ</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>6000</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add batch multi-image scanning, remove sample buttons, implement multi-sheet Excel management and weekly downloads
</commit_message>
<xml_diff>
--- a/ABA_Transactions_Latest.xlsx
+++ b/ABA_Transactions_Latest.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="ABA Transactions KHR" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Week_42_2026" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,4 +482,80 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Entry No</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>JV No</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Vendor / Customer / Employee</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Balance</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: resolve empty Excel download and ensure Week_3 multi-sheet rows persist properly
</commit_message>
<xml_diff>
--- a/ABA_Transactions_Latest.xlsx
+++ b/ABA_Transactions_Latest.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="ABA Transactions KHR" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Week_42_2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Week_3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -558,4 +559,172 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Entry No</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>JV No</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Vendor / Customer / Employee</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>57559</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>JV00605</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>57560</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>JV00606</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: resolve batch multi-scan dropping receipts, enable parallel AI analysis, and link active sheet to batch save
</commit_message>
<xml_diff>
--- a/ABA_Transactions_Latest.xlsx
+++ b/ABA_Transactions_Latest.xlsx
@@ -10,6 +10,7 @@
     <sheet name="ABA Transactions KHR" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Week_42_2026" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Week_3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Week_5" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -654,6 +655,170 @@
           <t>JV00605</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>57560</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>JV00606</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Entry No</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>JV No</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Vendor / Customer / Employee</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>57561</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>JV00607</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
@@ -662,12 +827,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+          <t>ហាងកាហ្វេ ជួបជុំ</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -684,7 +849,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -693,11 +858,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>57560</v>
+        <v>57562</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>JV00606</t>
+          <t>JV00608</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -708,12 +873,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+          <t>សេវាដឹកជញ្ជូន វីរៈប៊ុនថាំ</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+          <t>ថ្លៃផ្ញើអីវ៉ាន់</t>
         </is>
       </c>
       <c r="J3" t="n">
@@ -723,6 +888,52 @@
         <v>5000</v>
       </c>
       <c r="L3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>57563</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>JV00609</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ទិញក្រដាសការិយាល័យ</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>10000</v>
+      </c>
+      <c r="L4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(ocr): correct amount to 7500 KHR (.83) instead of 10000, add AI learning memory and smart normalization rule
</commit_message>
<xml_diff>
--- a/ABA_Transactions_Latest.xlsx
+++ b/ABA_Transactions_Latest.xlsx
@@ -3,10 +3,10 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="ABA Transactions KHR" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Week_42_2026" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Week_3" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Week_5" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Week_5" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ABA Transactions KHR" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Week_42_2026" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Week_3" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -450,20 +450,6 @@
   </sheetPr>
   <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6.83203125" customWidth="1" min="1" max="1"/>
-    <col width="14.83203125" customWidth="1" min="2" max="2"/>
-    <col width="10.83203125" customWidth="1" min="3" max="3"/>
-    <col width="12.83203125" customWidth="1" min="4" max="4"/>
-    <col width="12.83203125" customWidth="1" min="5" max="5"/>
-    <col width="14.83203125" customWidth="1" min="6" max="6"/>
-    <col width="14.83203125" customWidth="1" min="7" max="7"/>
-    <col width="32.83203125" customWidth="1" min="8" max="8"/>
-    <col width="30.83203125" customWidth="1" min="9" max="9"/>
-    <col width="12.83203125" customWidth="1" min="10" max="10"/>
-    <col width="12.83203125" customWidth="1" min="11" max="11"/>
-    <col width="12.83203125" customWidth="1" min="12" max="12"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -529,7 +515,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -542,11 +528,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>57560</v>
+        <v>57559</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>JV00606</t>
+          <t>JV00605</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -573,7 +559,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -586,11 +572,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>57559</v>
+        <v>57560</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>JV00605</t>
+          <t>JV00606</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -630,11 +616,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>57563</v>
+        <v>57561</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>JV00609</t>
+          <t>JV00607</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -644,24 +630,24 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
+          <t>ហាងកាហ្វេ ជួបជុំ</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ទិញក្រដាសការិយាល័យ</t>
+          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
         </is>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>10000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -705,7 +691,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -718,11 +704,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>57561</v>
+        <v>57563</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>JV00607</t>
+          <t>JV00609</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -732,19 +718,19 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>ហាងកាហ្វេ ជួបជុំ</t>
+          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
+          <t>ទិញក្រដាសការិយាល័យ</t>
         </is>
       </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>5000</v>
+        <v>7500</v>
       </c>
     </row>
   </sheetData>
@@ -753,6 +739,312 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Entry No</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>JV No</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Vendor / Customer / Employee</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>57559</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>JV00605</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>57560</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>JV00606</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>57561</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>JV00607</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ហាងកាហ្វេ ជួបជុំ</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>57562</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>JV00608</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>សេវាដឹកជញ្ជូន វីរៈប៊ុនថាំ</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>ថ្លៃផ្ញើអីវ៉ាន់</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>57563</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>JV00609</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>ទិញក្រដាសការិយាល័យ</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>7500</v>
+      </c>
+      <c r="L6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -842,7 +1134,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1018,310 +1310,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Entry No</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>JV No</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Vendor / Customer / Employee</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Debit</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>57559</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>JV00605</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>57560</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>JV00606</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>57561</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>JV00607</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>ហាងកាហ្វេ ជួបជុំ</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>57562</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>JV00608</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>សេវាដឹកជញ្ជូន វីរៈប៊ុនថាំ</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>ថ្លៃផ្ញើអីវ៉ាន់</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>57563</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>JV00609</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>ទិញក្រដាសការិយាល័យ</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="L6" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(order): count from bottom to top (No. 1 at bottom to No. 10 at top) and sync 10 rows in Week_5
</commit_message>
<xml_diff>
--- a/ABA_Transactions_Latest.xlsx
+++ b/ABA_Transactions_Latest.xlsx
@@ -1,7 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
     <sheet name="Week_5" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="ABA Transactions KHR" sheetId="2" state="visible" r:id="rId2"/>
@@ -9,6 +13,7 @@
     <sheet name="Week_3" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -20,7 +25,7 @@
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -48,9 +53,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -197,7 +202,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -232,7 +236,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -267,16 +270,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -398,46 +405,7 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -448,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,11 +483,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -528,13 +496,14 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>57559</v>
+        <v>57568</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>JV00605</t>
-        </is>
-      </c>
+          <t>JV02988</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -542,24 +511,25 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+          <t>KHAI NAM CO. LTD (សេវាបញ្ជូនឥវ៉ាន់)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
         </is>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>5000</v>
-      </c>
+        <v>16000</v>
+      </c>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -572,13 +542,14 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>57560</v>
+        <v>57567</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>JV00606</t>
-        </is>
-      </c>
+          <t>JV02987</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -586,28 +557,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+          <t>អ្នកលក់ទូទៅ (General Vendor)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+          <t>សម្ភារៈប្រើប្រាស់</t>
         </is>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>5000</v>
-      </c>
+        <v>56000</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -616,13 +588,14 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>57561</v>
+        <v>57566</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>JV00607</t>
-        </is>
-      </c>
+          <t>JV02986</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -630,28 +603,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>ហាងកាហ្វេ ជួបជុំ</t>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
         </is>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>5000</v>
-      </c>
+        <v>7500</v>
+      </c>
+      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -660,13 +634,14 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>57562</v>
+        <v>57565</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>JV00608</t>
-        </is>
-      </c>
+          <t>JV02985</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -674,12 +649,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>សេវាដឹកជញ្ជូន វីរៈប៊ុនថាំ</t>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (មាយ ណុយ)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>ថ្លៃផ្ញើអីវ៉ាន់</t>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -688,14 +663,15 @@
       <c r="K5" t="n">
         <v>5000</v>
       </c>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -704,13 +680,14 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>57563</v>
+        <v>57564</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>JV00609</t>
-        </is>
-      </c>
+          <t>JV00610</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -718,12 +695,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>ទិញក្រដាសការិយាល័យ</t>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -732,6 +709,237 @@
       <c r="K6" t="n">
         <v>7500</v>
       </c>
+      <c r="L6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>57563</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>JV00609</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ទិញក្រដាសការិយាល័យ</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>7500</v>
+      </c>
+      <c r="L7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>57562</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>JV00608</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>សេវាដឹកជញ្ជូន វីរៈប៊ុនថាំ</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ថ្លៃផ្ញើអីវ៉ាន់</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>57561</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>JV00607</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>ហាងកាហ្វេ ជួបជុំ</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>57560</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>JV00606</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>57559</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>JV00605</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -744,7 +952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -811,11 +1019,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -824,11 +1032,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>57559</v>
+        <v>57568</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>JV00605</t>
+          <t>JV02988</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -839,25 +1047,25 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+          <t>KHAI NAM CO. LTD (សេវាបញ្ជូនឥវ៉ាន់)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
         </is>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>5000</v>
+        <v>16000</v>
       </c>
       <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -870,11 +1078,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>57560</v>
+        <v>57567</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>JV00606</t>
+          <t>JV02987</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -885,29 +1093,29 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+          <t>អ្នកលក់ទូទៅ (General Vendor)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+          <t>សម្ភារៈប្រើប្រាស់</t>
         </is>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>5000</v>
+        <v>56000</v>
       </c>
       <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -916,11 +1124,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>57561</v>
+        <v>57566</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>JV00607</t>
+          <t>JV02986</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -931,29 +1139,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>ហាងកាហ្វេ ជួបជុំ</t>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
         </is>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>5000</v>
+        <v>7500</v>
       </c>
       <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -962,11 +1170,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>57562</v>
+        <v>57565</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>JV00608</t>
+          <t>JV02985</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -977,12 +1185,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>សេវាដឹកជញ្ជូន វីរៈប៊ុនថាំ</t>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (មាយ ណុយ)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>ថ្លៃផ្ញើអីវ៉ាន់</t>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -995,11 +1203,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1008,11 +1216,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>57563</v>
+        <v>57564</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>JV00609</t>
+          <t>JV00610</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -1023,12 +1231,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>ទិញក្រដាសការិយាល័យ</t>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -1038,6 +1246,236 @@
         <v>7500</v>
       </c>
       <c r="L6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>57563</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>JV00609</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ទិញក្រដាសការិយាល័យ</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>7500</v>
+      </c>
+      <c r="L7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>57562</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>JV00608</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>សេវាដឹកជញ្ជូន វីរៈប៊ុនថាំ</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ថ្លៃផ្ញើអីវ៉ាន់</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>57561</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>JV00607</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>ហាងកាហ្វេ ជួបជុំ</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>57560</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>JV00606</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>57559</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>JV00605</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1052,20 +1490,6 @@
   </sheetPr>
   <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6.83203125" customWidth="1" min="1" max="1"/>
-    <col width="14.83203125" customWidth="1" min="2" max="2"/>
-    <col width="10.83203125" customWidth="1" min="3" max="3"/>
-    <col width="12.83203125" customWidth="1" min="4" max="4"/>
-    <col width="12.83203125" customWidth="1" min="5" max="5"/>
-    <col width="14.83203125" customWidth="1" min="6" max="6"/>
-    <col width="14.83203125" customWidth="1" min="7" max="7"/>
-    <col width="32.83203125" customWidth="1" min="8" max="8"/>
-    <col width="30.83203125" customWidth="1" min="9" max="9"/>
-    <col width="12.83203125" customWidth="1" min="10" max="10"/>
-    <col width="12.83203125" customWidth="1" min="11" max="11"/>
-    <col width="12.83203125" customWidth="1" min="12" max="12"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1142,20 +1566,6 @@
   </sheetPr>
   <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6.83203125" customWidth="1" min="1" max="1"/>
-    <col width="14.83203125" customWidth="1" min="2" max="2"/>
-    <col width="10.83203125" customWidth="1" min="3" max="3"/>
-    <col width="12.83203125" customWidth="1" min="4" max="4"/>
-    <col width="12.83203125" customWidth="1" min="5" max="5"/>
-    <col width="14.83203125" customWidth="1" min="6" max="6"/>
-    <col width="14.83203125" customWidth="1" min="7" max="7"/>
-    <col width="32.83203125" customWidth="1" min="8" max="8"/>
-    <col width="30.83203125" customWidth="1" min="9" max="9"/>
-    <col width="12.83203125" customWidth="1" min="10" max="10"/>
-    <col width="12.83203125" customWidth="1" min="11" max="11"/>
-    <col width="12.83203125" customWidth="1" min="12" max="12"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1241,6 +1651,7 @@
           <t>JV00606</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -1262,6 +1673,7 @@
       <c r="K2" t="n">
         <v>5000</v>
       </c>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1285,6 +1697,7 @@
           <t>JV00605</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -1306,6 +1719,7 @@
       <c r="K3" t="n">
         <v>5000</v>
       </c>
+      <c r="L3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: rename ABA to All data, remove Week_5, and add 2026 12-month and 4-week dropdown selectors
</commit_message>
<xml_diff>
--- a/ABA_Transactions_Latest.xlsx
+++ b/ABA_Transactions_Latest.xlsx
@@ -7,70 +7,67 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ABA Transactions KHR" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Week_5" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026_M01_មករា" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="2026_M01_Week1" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="2026_M01_Week2" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="2026_M01_Week3" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="2026_M01_Week4" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="2026_M02_កុម្ភៈ" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="2026_M02_Week1" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="2026_M02_Week2" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="2026_M02_Week3" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="2026_M02_Week4" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="2026_M03_មីនា" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="2026_M03_Week1" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="2026_M03_Week2" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="2026_M03_Week3" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="2026_M03_Week4" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="2026_M04_មេសា" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="2026_M04_Week1" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="2026_M04_Week2" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="2026_M04_Week3" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="2026_M04_Week4" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="2026_M05_ឧសភា" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="2026_M05_Week1" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="2026_M05_Week2" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="2026_M05_Week3" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="2026_M05_Week4" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="2026_M06_មិថុនា" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="2026_M06_Week1" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="2026_M06_Week2" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="2026_M06_Week3" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="2026_M06_Week4" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="2026_M07_កក្កដា" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="2026_M07_Week1" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="2026_M07_Week2" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="2026_M07_Week3" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="2026_M07_Week4" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="2026_M08_សីហា" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="2026_M08_Week1" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="2026_M08_Week2" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="2026_M08_Week3" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="2026_M08_Week4" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="2026_M09_កញ្ញា" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="2026_M09_Week1" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="2026_M09_Week2" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="2026_M09_Week3" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="2026_M09_Week4" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="2026_M10_តុលា" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="2026_M10_Week1" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet name="2026_M10_Week2" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="2026_M10_Week3" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="2026_M10_Week4" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet name="2026_M11_វិច្ឆិកា" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet name="2026_M11_Week1" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet name="2026_M11_Week2" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet name="2026_M11_Week3" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet name="2026_M11_Week4" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet name="2026_M12_ធ្នូ" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet name="2026_M12_Week1" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet name="2026_M12_Week2" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet name="2026_M12_Week3" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet name="2026_M12_Week4" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet name="Week_42_2026" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet name="Week_3" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="All data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2026_M01_មករា" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2026_M01_Week1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2026_M01_Week2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026_M01_Week3" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2026_M01_Week4" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2026_M02_កុម្ភៈ" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2026_M02_Week1" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2026_M02_Week2" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="2026_M02_Week3" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="2026_M02_Week4" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="2026_M03_មីនា" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2026_M03_Week1" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="2026_M03_Week2" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="2026_M03_Week3" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="2026_M03_Week4" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="2026_M04_មេសា" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="2026_M04_Week1" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="2026_M04_Week2" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="2026_M04_Week3" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="2026_M04_Week4" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="2026_M05_ឧសភា" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="2026_M05_Week1" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="2026_M05_Week2" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="2026_M05_Week3" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="2026_M05_Week4" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="2026_M06_មិថុនា" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="2026_M06_Week1" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="2026_M06_Week2" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="2026_M06_Week3" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="2026_M06_Week4" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="2026_M07_កក្កដា" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="2026_M07_Week1" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="2026_M07_Week2" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="2026_M07_Week3" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="2026_M07_Week4" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="2026_M08_សីហា" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="2026_M08_Week1" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="2026_M08_Week2" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="2026_M08_Week3" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="2026_M08_Week4" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="2026_M09_កញ្ញា" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="2026_M09_Week1" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="2026_M09_Week2" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="2026_M09_Week3" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="2026_M09_Week4" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="2026_M10_តុលា" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="2026_M10_Week1" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="2026_M10_Week2" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="2026_M10_Week3" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="2026_M10_Week4" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="2026_M11_វិច្ឆិកា" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="2026_M11_Week1" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="2026_M11_Week2" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="2026_M11_Week3" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="2026_M11_Week4" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="2026_M12_ធ្នូ" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="2026_M12_Week1" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="2026_M12_Week2" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="2026_M12_Week3" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="2026_M12_Week4" sheetId="61" state="visible" r:id="rId61"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -563,7 +560,6 @@
           <t>JV02988</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -585,7 +581,6 @@
       <c r="K2" t="n">
         <v>16000</v>
       </c>
-      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -609,7 +604,6 @@
           <t>JV02987</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -631,7 +625,6 @@
       <c r="K3" t="n">
         <v>56000</v>
       </c>
-      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -655,7 +648,6 @@
           <t>JV02986</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -677,7 +669,6 @@
       <c r="K4" t="n">
         <v>7500</v>
       </c>
-      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -701,7 +692,6 @@
           <t>JV02985</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -723,7 +713,6 @@
       <c r="K5" t="n">
         <v>5000</v>
       </c>
-      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -747,7 +736,6 @@
           <t>JV00610</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -769,7 +757,6 @@
       <c r="K6" t="n">
         <v>7500</v>
       </c>
-      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -793,7 +780,6 @@
           <t>JV00609</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -815,7 +801,6 @@
       <c r="K7" t="n">
         <v>7500</v>
       </c>
-      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -839,7 +824,6 @@
           <t>JV00608</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -861,7 +845,6 @@
       <c r="K8" t="n">
         <v>5000</v>
       </c>
-      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -885,7 +868,6 @@
           <t>JV00607</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -907,7 +889,6 @@
       <c r="K9" t="n">
         <v>5000</v>
       </c>
-      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -931,7 +912,6 @@
           <t>JV00606</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -953,7 +933,6 @@
       <c r="K10" t="n">
         <v>5000</v>
       </c>
-      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -977,7 +956,6 @@
           <t>JV00605</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -999,7 +977,6 @@
       <c r="K11" t="n">
         <v>5000</v>
       </c>
-      <c r="L11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1012,7 +989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1075,6 +1052,50 @@
         <is>
           <t>Balance</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>57568</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>JV02988</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>KHAI NAM CO. LTD (សេវាបញ្ជូនឥវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>16000</v>
       </c>
     </row>
   </sheetData>
@@ -1088,7 +1109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1152,52 +1173,6 @@
           <t>Balance</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-02-16</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>57568</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>JV02988</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>KHAI NAM CO. LTD (សេវាបញ្ជូនឥវ៉ាន់)</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>16000</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1818,7 +1793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1882,466 +1857,6 @@
           <t>Balance</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-02-16</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>57568</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>JV02988</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>KHAI NAM CO. LTD (សេវាបញ្ជូនឥវ៉ាន់)</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>16000</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>9</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>57567</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>JV02987</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>អ្នកលក់ទូទៅ (General Vendor)</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>សម្ភារៈប្រើប្រាស់</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>56000</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>57566</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>JV02986</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>7500</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>57565</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>JV02985</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>សេវាបញ្ជូនឥវ៉ាន់ (មាយ ណុយ)</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>57564</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>JV00610</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>7500</v>
-      </c>
-      <c r="L6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>57563</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>JV00609</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>ទិញក្រដាសការិយាល័យ</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>7500</v>
-      </c>
-      <c r="L7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>57562</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>JV00608</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>សេវាដឹកជញ្ជូន វីរៈប៊ុនថាំ</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>ថ្លៃផ្ញើអីវ៉ាន់</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>57561</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>JV00607</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>ហាងកាហ្វេ ជួបជុំ</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>2</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>57560</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>JV00606</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>57559</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>JV00605</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4178,7 +3693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4241,6 +3756,270 @@
         <is>
           <t>Balance</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>57567</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>JV02987</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>អ្នកលក់ទូទៅ (General Vendor)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>សម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>56000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>57566</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>JV02986</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>57565</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>JV02985</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (មាយ ណុយ)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>57564</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>JV00610</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>57560</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>JV00606</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>57559</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>JV00605</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>5000</v>
       </c>
     </row>
   </sheetData>
@@ -4254,7 +4033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4318,282 +4097,6 @@
           <t>Balance</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>57567</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>JV02987</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>អ្នកលក់ទូទៅ (General Vendor)</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>សម្ភារៈប្រើប្រាស់</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>56000</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>57566</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>JV02986</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>7500</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>57565</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>JV02985</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>សេវាបញ្ជូនឥវ៉ាន់ (មាយ ណុយ)</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>57564</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>JV00610</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>7500</v>
-      </c>
-      <c r="L5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>57560</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>JV00606</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>57559</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>JV00605</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4682,7 +4185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4745,6 +4248,226 @@
         <is>
           <t>Balance</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>57567</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>JV02987</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>អ្នកលក់ទូទៅ (General Vendor)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>សម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>56000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>57566</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>JV02986</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>57564</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>JV00610</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>57560</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>JV00606</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>57559</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>JV00605</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>5000</v>
       </c>
     </row>
   </sheetData>
@@ -4758,7 +4481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4825,11 +4548,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4838,14 +4561,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>57567</v>
+        <v>57565</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>JV02987</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>JV02985</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -4853,205 +4575,20 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>អ្នកលក់ទូទៅ (General Vendor)</t>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (មាយ ណុយ)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>សម្ភារៈប្រើប្រាស់</t>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
         </is>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>56000</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>4</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>57566</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>JV02986</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>7500</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>57564</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>JV00610</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>7500</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>57560</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>JV00606</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
         <v>5000</v>
       </c>
-      <c r="L5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>57559</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>JV00605</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5064,7 +4601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5131,11 +4668,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -5144,14 +4681,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>57565</v>
+        <v>57563</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>JV02985</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>JV00609</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -5159,21 +4695,108 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>សេវាបញ្ជូនឥវ៉ាន់ (មាយ ណុយ)</t>
+          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+          <t>ទិញក្រដាសការិយាល័យ</t>
         </is>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>57562</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>JV00608</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>សេវាដឹកជញ្ជូន វីរៈប៊ុនថាំ</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ថ្លៃផ្ញើអីវ៉ាន់</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
         <v>5000</v>
       </c>
-      <c r="L2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>57561</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>JV00607</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ហាងកាហ្វេ ជួបជុំ</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5000</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5186,7 +4809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5250,144 +4873,6 @@
           <t>Balance</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>57563</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>JV00609</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>ទិញក្រដាសការិយាល័យ</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>7500</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>57562</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>JV00608</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>សេវាដឹកជញ្ជូន វីរៈប៊ុនថាំ</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>ថ្លៃផ្ញើអីវ៉ាន់</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>57561</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>JV00607</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>ហាងកាហ្វេ ជួបជុំ</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5552,7 +5037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5615,6 +5100,138 @@
         <is>
           <t>Balance</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>57563</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>JV00609</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ទិញក្រដាសការិយាល័យ</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>57562</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>JV00608</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>សេវាដឹកជញ្ជូន វីរៈប៊ុនថាំ</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ថ្លៃផ្ញើអីវ៉ាន់</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>57561</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>JV00607</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ហាងកាហ្វេ ជួបជុំ</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5000</v>
       </c>
     </row>
   </sheetData>
@@ -5628,7 +5245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5692,144 +5309,6 @@
           <t>Balance</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>57563</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>JV00609</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>ទិញក្រដាសការិយាល័យ</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>7500</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>57562</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>JV00608</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>សេវាដឹកជញ្ជូន វីរៈប៊ុនថាំ</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>ថ្លៃផ្ញើអីវ៉ាន់</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>57561</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>JV00607</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>ហាងកាហ្វេ ជួបជុំ</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6672,333 +6151,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Entry No</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>JV No</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Vendor / Customer / Employee</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Debit</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Balance</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Entry No</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>JV No</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Vendor / Customer / Employee</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Debit</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Balance</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Entry No</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>JV No</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Vendor / Customer / Employee</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Debit</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>57560</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>JV00606</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>57559</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>JV00605</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7061,6 +6220,50 @@
         <is>
           <t>Balance</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>57568</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>JV02988</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>KHAI NAM CO. LTD (សេវាបញ្ជូនឥវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>16000</v>
       </c>
     </row>
   </sheetData>
@@ -7074,7 +6277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7138,52 +6341,6 @@
           <t>Balance</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-02-16</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>57568</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>JV02988</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>KHAI NAM CO. LTD (សេវាបញ្ជូនឥវ៉ាន់)</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>16000</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: remember entry date for auto sheet routing and preserve paper receipt date in excel
</commit_message>
<xml_diff>
--- a/ABA_Transactions_Latest.xlsx
+++ b/ABA_Transactions_Latest.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -540,11 +540,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -553,11 +553,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>57568</v>
+        <v>57559</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>JV02988</t>
+          <t>JV00605</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -567,24 +567,24 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>KHAI NAM CO. LTD (សេវាបញ្ជូនឥវ៉ាន់)</t>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
         </is>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>16000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -597,11 +597,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>57567</v>
+        <v>57560</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>JV02987</t>
+          <t>JV00606</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -611,28 +611,28 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>អ្នកលក់ទូទៅ (General Vendor)</t>
+          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>សម្ភារៈប្រើប្រាស់</t>
+          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
         </is>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>56000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -641,11 +641,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>57566</v>
+        <v>57561</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>JV02986</t>
+          <t>JV00607</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -655,28 +655,28 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
+          <t>ហាងកាហ្វេ ជួបជុំ</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
         </is>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>7500</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -685,11 +685,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>57565</v>
+        <v>57562</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>JV02985</t>
+          <t>JV00608</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -699,12 +699,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>សេវាបញ្ជូនឥវ៉ាន់ (មាយ ណុយ)</t>
+          <t>សេវាដឹកជញ្ជូន វីរៈប៊ុនថាំ</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+          <t>ថ្លៃផ្ញើអីវ៉ាន់</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -716,11 +716,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -729,11 +729,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>57564</v>
+        <v>57563</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>JV00610</t>
+          <t>JV00609</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -743,12 +743,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
+          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+          <t>ទិញក្រដាសការិយាល័យ</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -760,11 +760,11 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -773,11 +773,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>57563</v>
+        <v>57564</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>JV00609</t>
+          <t>JV00610</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -787,12 +787,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>ទិញក្រដាសការិយាល័យ</t>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -804,11 +804,11 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -817,11 +817,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>57562</v>
+        <v>57565</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>JV00608</t>
+          <t>JV02985</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>សេវាដឹកជញ្ជូន វីរៈប៊ុនថាំ</t>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (មាយ ណុយ)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>ថ្លៃផ្ញើអីវ៉ាន់</t>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -848,11 +848,11 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>57561</v>
+        <v>57566</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>JV00607</t>
+          <t>JV02986</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -875,24 +875,24 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>ហាងកាហ្វេ ជួបជុំ</t>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
         </is>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>5000</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -905,11 +905,11 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>57560</v>
+        <v>57567</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>JV00606</t>
+          <t>JV02987</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -919,28 +919,28 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+          <t>អ្នកលក់ទូទៅ (General Vendor)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+          <t>សម្ភារៈប្រើប្រាស់</t>
         </is>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>5000</v>
+        <v>56000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -949,11 +949,11 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>57559</v>
+        <v>57568</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>JV00605</t>
+          <t>JV02988</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -963,19 +963,68 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>ខេមា គ្លីនិក &amp; ដេនថល (Khema Clinic)</t>
+          <t>KHAI NAM CO. LTD (សេវាបញ្ជូនឥវ៉ាន់)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ទិញសម្ភារៈប្រើប្រាស់</t>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
         </is>
       </c>
       <c r="J11" t="n">
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>5000</v>
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>57569</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>JV02989</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>INV-TEST-ROUTE-1</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>ហាងសាកល្បង Auto Date</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>សេវាដឹកជញ្ជូន</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>7500</v>
       </c>
     </row>
   </sheetData>
@@ -4601,7 +4650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4668,7 +4717,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -4681,11 +4730,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>57563</v>
+        <v>57561</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>JV00609</t>
+          <t>JV00607</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -4695,19 +4744,19 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
+          <t>ហាងកាហ្វេ ជួបជុំ</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ទិញក្រដាសការិយាល័យ</t>
+          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
         </is>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>7500</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="3">
@@ -4756,7 +4805,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -4769,11 +4818,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>57561</v>
+        <v>57563</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>JV00607</t>
+          <t>JV00609</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -4783,19 +4832,68 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>ហាងកាហ្វេ ជួបជុំ</t>
+          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
+          <t>ទិញក្រដាសការិយាល័យ</t>
         </is>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>5000</v>
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>57569</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>JV02989</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>INV-TEST-ROUTE-1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>ហាងសាកល្បង Auto Date</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>សេវាដឹកជញ្ជូន</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>7500</v>
       </c>
     </row>
   </sheetData>
@@ -4809,7 +4907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4873,6 +4971,56 @@
           <t>Balance</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>57569</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>JV02989</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>INV-TEST-ROUTE-1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>ហាងសាកល្បង Auto Date</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>សេវាដឹកជញ្ជូន</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>7500</v>
+      </c>
+      <c r="L2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: restore 4 entries entered yesterday with entryDate 2026-10-20 and populate October sheets
</commit_message>
<xml_diff>
--- a/ABA_Transactions_Latest.xlsx
+++ b/ABA_Transactions_Latest.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,6 +560,7 @@
           <t>JV00605</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -604,6 +605,7 @@
           <t>JV00606</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -648,6 +650,7 @@
           <t>JV00607</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -692,6 +695,7 @@
           <t>JV00608</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -736,6 +740,7 @@
           <t>JV00609</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -780,6 +785,7 @@
           <t>JV00610</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -824,6 +830,7 @@
           <t>JV02985</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -868,6 +875,7 @@
           <t>JV02986</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -912,6 +920,7 @@
           <t>JV02987</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -956,6 +965,7 @@
           <t>JV02988</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -976,55 +986,6 @@
       </c>
       <c r="K11" t="n">
         <v>16000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>57569</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>JV02989</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>INV-TEST-ROUTE-1</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>ហាងសាកល្បង Auto Date</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>សេវាដឹកជញ្ជូន</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
-        <v>7500</v>
       </c>
     </row>
   </sheetData>
@@ -4650,7 +4611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4737,6 +4698,7 @@
           <t>JV00607</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -4781,6 +4743,7 @@
           <t>JV00608</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -4825,6 +4788,7 @@
           <t>JV00609</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -4853,7 +4817,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4862,18 +4826,14 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>57569</v>
+        <v>57565</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>JV02989</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>INV-TEST-ROUTE-1</t>
-        </is>
-      </c>
+          <t>JV02985</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -4881,19 +4841,154 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>ហាងសាកល្បង Auto Date</t>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (មាយ ណុយ)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>សេវាដឹកជញ្ជូន</t>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
         </is>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>57566</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>JV02986</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
         <v>7500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>57567</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>JV02987</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>អ្នកលក់ទូទៅ (General Vendor)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>សម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>56000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>57568</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>JV02988</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>KHAI NAM CO. LTD (សេវាបញ្ជូនឥវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>16000</v>
       </c>
     </row>
   </sheetData>
@@ -4907,7 +5002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4971,56 +5066,6 @@
           <t>Balance</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GL-JE</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>57569</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>JV02989</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>INV-TEST-ROUTE-1</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>KHEMA88888</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>ហាងសាកល្បង Auto Date</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>សេវាដឹកជញ្ជូន</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>7500</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5185,7 +5230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5252,7 +5297,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -5265,13 +5310,14 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>57563</v>
+        <v>57561</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>JV00609</t>
-        </is>
-      </c>
+          <t>JV00607</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -5279,19 +5325,19 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
+          <t>ហាងកាហ្វេ ជួបជុំ</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ទិញក្រដាសការិយាល័យ</t>
+          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
         </is>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>7500</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="3">
@@ -5316,6 +5362,7 @@
           <t>JV00608</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -5340,7 +5387,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -5353,13 +5400,14 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>57561</v>
+        <v>57563</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>JV00607</t>
-        </is>
-      </c>
+          <t>JV00609</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>KHEMA88888</t>
@@ -5367,19 +5415,199 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>ហាងកាហ្វេ ជួបជុំ</t>
+          <t>សម្ភារៈការិយាល័យ ភ្នំពេញ</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ទិញសម្ភារៈ និងកាហ្វេ</t>
+          <t>ទិញក្រដាសការិយាល័យ</t>
         </is>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>57565</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>JV02985</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (មាយ ណុយ)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
         <v>5000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>57566</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>JV02986</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>សេវាបញ្ជូនឥវ៉ាន់ (Manit)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>57567</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>JV02987</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>អ្នកលក់ទូទៅ (General Vendor)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>សម្ភារៈប្រើប្រាស់</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>56000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GL-JE</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>57568</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>JV02988</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>KHEMA88888</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>KHAI NAM CO. LTD (សេវាបញ្ជូនឥវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ថ្លៃសេវាទូទៅ (ថ្លៃផ្ញើអីវ៉ាន់)</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>16000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>